<commit_message>
Agregar enlaces en TAG_RESOURCES.xlsx (7 TAGs, 9 enlaces)
Specifications / Handbook_Manual / Maintenance llenados a mano con Ctrl+K.
Fuente alineada con el sitio publicado en commit 3d98060.
</commit_message>
<xml_diff>
--- a/TAG_RESOURCES.xlsx
+++ b/TAG_RESOURCES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\administrador\google-sites-migrator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8019C00-6175-41C3-9688-7DBAE7FFE56D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC9158C-42EC-44FC-A788-F280FDDB32A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
   <si>
     <t>TAG_ID</t>
   </si>
@@ -161,6 +161,12 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1yWg0gxxrTn9aG0JBJuClnerLCuVxGveX/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1GP_5peG1Kz38IixfG8e5zMKi0f_HLmsc/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1b1tp5_6Qi-BCIRfIfDii_a57OacD5pH2/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
@@ -240,7 +246,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -248,7 +254,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -558,6 +563,7 @@
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="88.85546875" customWidth="1"/>
     <col min="3" max="4" width="30" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -588,7 +594,9 @@
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" s="3" t="s">
+        <v>47</v>
+      </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
     </row>
@@ -611,11 +619,23 @@
       <c r="A8" t="s">
         <v>10</v>
       </c>
+      <c r="B8" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
+      <c r="B9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -777,7 +797,7 @@
       <c r="A40" t="s">
         <v>42</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="3" t="s">
         <v>44</v>
       </c>
     </row>
@@ -785,7 +805,7 @@
       <c r="A41" t="s">
         <v>43</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="3" t="s">
         <v>46</v>
       </c>
     </row>
@@ -795,6 +815,9 @@
     <hyperlink ref="B35" r:id="rId2" xr:uid="{FB6D2F31-4695-4A27-BEBD-E9AA844A45DA}"/>
     <hyperlink ref="B36" r:id="rId3" xr:uid="{3DEA2B13-70A9-49BE-AB09-2E8AA32CD8D0}"/>
     <hyperlink ref="B41" r:id="rId4" xr:uid="{85D92C4D-ED09-41B4-9708-E56296EC1047}"/>
+    <hyperlink ref="B4" r:id="rId5" xr:uid="{808FCD4A-3A3E-4A66-8155-420CC239F6FB}"/>
+    <hyperlink ref="B8" r:id="rId6" xr:uid="{32F4ED13-A7FE-4C0B-A2C4-F519A19A1ABE}"/>
+    <hyperlink ref="B9" r:id="rId7" xr:uid="{6DBECEFE-189D-4559-8948-76E3F72B0918}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Manuales y especificaciones adicionados
</commit_message>
<xml_diff>
--- a/TAG_RESOURCES.xlsx
+++ b/TAG_RESOURCES.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30120"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\administrador\google-sites-migrator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC9158C-42EC-44FC-A788-F280FDDB32A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15A99A8C-FF94-4D64-B058-4D6379282E8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TAG_RESOURCES" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
   <si>
     <t>TAG_ID</t>
   </si>
@@ -167,6 +180,21 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1b1tp5_6Qi-BCIRfIfDii_a57OacD5pH2/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1VlvZySZLnHyeeEJD8dx4-j0sjiE2PmyI/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1w5nv_m9gUF5V6tVU1n1bx2inkPnPzgEq/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1UGFMRq50zcTrQDKkIio8FFdHR2fhSnYd/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Ww5Pe2vGCYdbdcHhLhntFV3eON3Z3S36/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1hDeqqyd7533etrn4FxXP4158a9O9bxuD/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
@@ -604,16 +632,25 @@
       <c r="A5" t="s">
         <v>7</v>
       </c>
+      <c r="B5" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
+      <c r="B6" s="3" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
+      <c r="B7" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -672,97 +709,106 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B28" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B29" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B34" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>37</v>
       </c>
@@ -770,7 +816,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>38</v>
       </c>
@@ -778,22 +824,34 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B37" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B38" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B39" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>42</v>
       </c>
@@ -801,7 +859,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>43</v>
       </c>
@@ -818,6 +876,14 @@
     <hyperlink ref="B4" r:id="rId5" xr:uid="{808FCD4A-3A3E-4A66-8155-420CC239F6FB}"/>
     <hyperlink ref="B8" r:id="rId6" xr:uid="{32F4ED13-A7FE-4C0B-A2C4-F519A19A1ABE}"/>
     <hyperlink ref="B9" r:id="rId7" xr:uid="{6DBECEFE-189D-4559-8948-76E3F72B0918}"/>
+    <hyperlink ref="B39" r:id="rId8" xr:uid="{AB547736-CF83-4724-98E0-DA894B00D043}"/>
+    <hyperlink ref="C39" r:id="rId9" xr:uid="{CA06C4F9-F00E-4A86-AC4B-FE2129626221}"/>
+    <hyperlink ref="B38" r:id="rId10" xr:uid="{3C010399-0B4B-4ECD-BE2A-F85C167CBDC9}"/>
+    <hyperlink ref="B34" r:id="rId11" xr:uid="{1D04FA18-E9D6-481A-8354-A00B411C342B}"/>
+    <hyperlink ref="B37" r:id="rId12" xr:uid="{12ADA2CB-339D-470E-A564-3F43133F5225}"/>
+    <hyperlink ref="B5" r:id="rId13" xr:uid="{9A47915E-3AA1-4499-A8F2-9DB02A794A3C}"/>
+    <hyperlink ref="B28" r:id="rId14" xr:uid="{00EB2E8B-5029-4E83-BDEC-AEF74250CC01}"/>
+    <hyperlink ref="B29" r:id="rId15" xr:uid="{A186D904-9D71-4AEF-A675-39C58008A8B0}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>